<commit_message>
Expanded visualization metrics and added ranking features
</commit_message>
<xml_diff>
--- a/outputs/space_syntax_summary.xlsx
+++ b/outputs/space_syntax_summary.xlsx
@@ -519,10 +519,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.982891</v>
+        <v>0.982837</v>
       </c>
       <c r="C3" t="n">
-        <v>0.856363</v>
+        <v>0.859103</v>
       </c>
       <c r="D3" t="n">
         <v>1.000216</v>
@@ -531,24 +531,24 @@
         <v>0.83127</v>
       </c>
       <c r="F3" t="n">
-        <v>0.986124</v>
+        <v>0.98608</v>
       </c>
       <c r="G3" t="n">
-        <v>0.834914</v>
+        <v>0.8375860000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>90.8939</v>
+        <v>90.25060000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>0.613617</v>
+        <v>0.6179480000000001</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>3.9412e-66</t>
+          <t>4.3261e-67</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>94.42</v>
+        <v>94.72</v>
       </c>
     </row>
     <row r="4">
@@ -636,36 +636,36 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.023949</v>
+        <v>1.018954</v>
       </c>
       <c r="C6" t="n">
-        <v>0.820013</v>
+        <v>0.825339</v>
       </c>
       <c r="D6" t="n">
-        <v>1.006552</v>
+        <v>1.005853</v>
       </c>
       <c r="E6" t="n">
-        <v>0.820483</v>
+        <v>0.818847</v>
       </c>
       <c r="F6" t="n">
-        <v>1.019479</v>
+        <v>1.015406</v>
       </c>
       <c r="G6" t="n">
-        <v>0.805449</v>
+        <v>0.809887</v>
       </c>
       <c r="H6" t="n">
-        <v>81.98560000000001</v>
+        <v>78.7542</v>
       </c>
       <c r="I6" t="n">
-        <v>0.544669</v>
+        <v>0.5585020000000001</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1.0768e-60</t>
+          <t>7.1101e-64</t>
         </is>
       </c>
       <c r="K6" t="n">
-        <v>94.03</v>
+        <v>94.5</v>
       </c>
     </row>
     <row r="7">
@@ -714,36 +714,36 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.16817</v>
+        <v>1.164951</v>
       </c>
       <c r="C8" t="n">
-        <v>0.86758</v>
+        <v>0.868475</v>
       </c>
       <c r="D8" t="n">
-        <v>1.035505</v>
+        <v>1.034806</v>
       </c>
       <c r="E8" t="n">
-        <v>0.829651</v>
+        <v>0.827832</v>
       </c>
       <c r="F8" t="n">
-        <v>1.129437</v>
+        <v>1.12681</v>
       </c>
       <c r="G8" t="n">
-        <v>0.848445</v>
+        <v>0.8489640000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>77.8249</v>
+        <v>76.9564</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6522210000000001</v>
+        <v>0.657346</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>3.5174e-133</t>
+          <t>2.3977e-135</t>
         </is>
       </c>
       <c r="K8" t="n">
-        <v>96.88</v>
+        <v>97.05</v>
       </c>
     </row>
     <row r="9">
@@ -792,36 +792,36 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.176377</v>
+        <v>1.168457</v>
       </c>
       <c r="C10" t="n">
-        <v>0.842465</v>
+        <v>0.845939</v>
       </c>
       <c r="D10" t="n">
-        <v>1.046597</v>
+        <v>1.045629</v>
       </c>
       <c r="E10" t="n">
-        <v>0.849468</v>
+        <v>0.8469179999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>1.138944</v>
+        <v>1.132538</v>
       </c>
       <c r="G10" t="n">
-        <v>0.828537</v>
+        <v>0.831207</v>
       </c>
       <c r="H10" t="n">
-        <v>83.2325</v>
+        <v>80.3133</v>
       </c>
       <c r="I10" t="n">
-        <v>0.604552</v>
+        <v>0.6210639999999999</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>1.5042e-94</t>
+          <t>2.6678e-100</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>93.70999999999999</v>
+        <v>94.09</v>
       </c>
     </row>
     <row r="11">
@@ -831,36 +831,36 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.04675</v>
+        <v>1.001214</v>
       </c>
       <c r="C11" t="n">
-        <v>0.818062</v>
+        <v>0.820234</v>
       </c>
       <c r="D11" t="n">
-        <v>1.004171</v>
+        <v>1.000381</v>
       </c>
       <c r="E11" t="n">
-        <v>0.828778</v>
+        <v>0.818209</v>
       </c>
       <c r="F11" t="n">
-        <v>1.032423</v>
+        <v>0.998318</v>
       </c>
       <c r="G11" t="n">
-        <v>0.804701</v>
+        <v>0.803427</v>
       </c>
       <c r="H11" t="n">
-        <v>83.63720000000001</v>
+        <v>80.1497</v>
       </c>
       <c r="I11" t="n">
-        <v>0.604276</v>
+        <v>0.598837</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>7.0869e-73</t>
+          <t>4.7676e-69</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>93.33</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -870,36 +870,36 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.282495</v>
+        <v>1.28105</v>
       </c>
       <c r="C12" t="n">
-        <v>0.888439</v>
+        <v>0.891085</v>
       </c>
       <c r="D12" t="n">
-        <v>1.029612</v>
+        <v>1.029276</v>
       </c>
       <c r="E12" t="n">
-        <v>0.838544</v>
+        <v>0.837365</v>
       </c>
       <c r="F12" t="n">
-        <v>1.208994</v>
+        <v>1.207694</v>
       </c>
       <c r="G12" t="n">
-        <v>0.86311</v>
+        <v>0.864987</v>
       </c>
       <c r="H12" t="n">
-        <v>69.61069999999999</v>
+        <v>68.9392</v>
       </c>
       <c r="I12" t="n">
-        <v>0.638305</v>
+        <v>0.6464530000000001</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>6.8141e-140</t>
+          <t>6.9671e-144</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>95.88</v>
+        <v>96.03</v>
       </c>
     </row>
     <row r="13">
@@ -1026,36 +1026,36 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.932376</v>
+        <v>0.912093</v>
       </c>
       <c r="C16" t="n">
-        <v>0.846079</v>
+        <v>0.844958</v>
       </c>
       <c r="D16" t="n">
-        <v>0.969094</v>
+        <v>0.964915</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8215249999999999</v>
+        <v>0.813822</v>
       </c>
       <c r="F16" t="n">
-        <v>0.942622</v>
+        <v>0.926789</v>
       </c>
       <c r="G16" t="n">
-        <v>0.829029</v>
+        <v>0.826648</v>
       </c>
       <c r="H16" t="n">
-        <v>75.1554</v>
+        <v>71.64230000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>0.420558</v>
+        <v>0.424485</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>1.2830e-54</t>
+          <t>9.2284e-55</t>
         </is>
       </c>
       <c r="K16" t="n">
-        <v>96.06999999999999</v>
+        <v>96.33</v>
       </c>
     </row>
     <row r="17">
@@ -1104,36 +1104,36 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1.125226</v>
+        <v>1.120469</v>
       </c>
       <c r="C18" t="n">
-        <v>0.823987</v>
+        <v>0.825168</v>
       </c>
       <c r="D18" t="n">
-        <v>1.033952</v>
+        <v>1.03251</v>
       </c>
       <c r="E18" t="n">
-        <v>0.825287</v>
+        <v>0.821533</v>
       </c>
       <c r="F18" t="n">
-        <v>1.098088</v>
+        <v>1.094084</v>
       </c>
       <c r="G18" t="n">
-        <v>0.810383</v>
+        <v>0.810469</v>
       </c>
       <c r="H18" t="n">
-        <v>72.5958</v>
+        <v>70.5129</v>
       </c>
       <c r="I18" t="n">
-        <v>0.6029369999999999</v>
+        <v>0.612317</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>9.0817e-115</t>
+          <t>2.3251e-118</t>
         </is>
       </c>
       <c r="K18" t="n">
-        <v>94.34999999999999</v>
+        <v>94.48</v>
       </c>
     </row>
     <row r="19">
@@ -1143,36 +1143,36 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1.109865</v>
+        <v>1.105436</v>
       </c>
       <c r="C19" t="n">
-        <v>0.8438099999999999</v>
+        <v>0.8448020000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>1.027018</v>
+        <v>1.025996</v>
       </c>
       <c r="E19" t="n">
-        <v>0.846346</v>
+        <v>0.84391</v>
       </c>
       <c r="F19" t="n">
-        <v>1.084396</v>
+        <v>1.080767</v>
       </c>
       <c r="G19" t="n">
-        <v>0.827987</v>
+        <v>0.82846</v>
       </c>
       <c r="H19" t="n">
-        <v>80.6808</v>
+        <v>79.4636</v>
       </c>
       <c r="I19" t="n">
-        <v>0.633592</v>
+        <v>0.640931</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>7.6678e-101</t>
+          <t>3.4689e-103</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>93.47</v>
+        <v>93.65000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1182,36 +1182,36 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.039049</v>
+        <v>1.026574</v>
       </c>
       <c r="C20" t="n">
-        <v>0.811775</v>
+        <v>0.812183</v>
       </c>
       <c r="D20" t="n">
-        <v>1.032437</v>
+        <v>1.030277</v>
       </c>
       <c r="E20" t="n">
-        <v>0.829803</v>
+        <v>0.825429</v>
       </c>
       <c r="F20" t="n">
-        <v>1.035773</v>
+        <v>1.026036</v>
       </c>
       <c r="G20" t="n">
-        <v>0.7987300000000001</v>
+        <v>0.798495</v>
       </c>
       <c r="H20" t="n">
-        <v>93.5778</v>
+        <v>89.3182</v>
       </c>
       <c r="I20" t="n">
-        <v>0.591038</v>
+        <v>0.602822</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>1.4672e-68</t>
+          <t>1.4156e-70</t>
         </is>
       </c>
       <c r="K20" t="n">
-        <v>92.59</v>
+        <v>92.87</v>
       </c>
     </row>
     <row r="21">
@@ -1221,36 +1221,36 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.139848</v>
+        <v>1.13369</v>
       </c>
       <c r="C21" t="n">
-        <v>0.840526</v>
+        <v>0.840616</v>
       </c>
       <c r="D21" t="n">
-        <v>0.9972569999999999</v>
+        <v>0.9964499999999999</v>
       </c>
       <c r="E21" t="n">
-        <v>0.822966</v>
+        <v>0.820837</v>
       </c>
       <c r="F21" t="n">
-        <v>1.098615</v>
+        <v>1.093867</v>
       </c>
       <c r="G21" t="n">
-        <v>0.82156</v>
+        <v>0.82128</v>
       </c>
       <c r="H21" t="n">
-        <v>86.62430000000001</v>
+        <v>84.68510000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>0.599204</v>
+        <v>0.603159</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>5.6811e-150</t>
+          <t>9.2467e-152</t>
         </is>
       </c>
       <c r="K21" t="n">
-        <v>94.45</v>
+        <v>94.56</v>
       </c>
     </row>
     <row r="22">
@@ -1260,36 +1260,36 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1.037293</v>
+        <v>1.031112</v>
       </c>
       <c r="C22" t="n">
-        <v>0.803509</v>
+        <v>0.805455</v>
       </c>
       <c r="D22" t="n">
-        <v>1.002796</v>
+        <v>1.001313</v>
       </c>
       <c r="E22" t="n">
-        <v>0.805621</v>
+        <v>0.803164</v>
       </c>
       <c r="F22" t="n">
-        <v>1.027319</v>
+        <v>1.022372</v>
       </c>
       <c r="G22" t="n">
-        <v>0.789957</v>
+        <v>0.791022</v>
       </c>
       <c r="H22" t="n">
-        <v>85.9443</v>
+        <v>82.62090000000001</v>
       </c>
       <c r="I22" t="n">
-        <v>0.60112</v>
+        <v>0.61009</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>8.2628e-90</t>
+          <t>2.9209e-92</t>
         </is>
       </c>
       <c r="K22" t="n">
-        <v>94.13</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="23">
@@ -1299,36 +1299,36 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.196855</v>
+        <v>1.182321</v>
       </c>
       <c r="C23" t="n">
-        <v>0.878571</v>
+        <v>0.878296</v>
       </c>
       <c r="D23" t="n">
-        <v>1.054234</v>
+        <v>1.053014</v>
       </c>
       <c r="E23" t="n">
-        <v>0.8634230000000001</v>
+        <v>0.860187</v>
       </c>
       <c r="F23" t="n">
-        <v>1.153824</v>
+        <v>1.14287</v>
       </c>
       <c r="G23" t="n">
-        <v>0.858835</v>
+        <v>0.858139</v>
       </c>
       <c r="H23" t="n">
-        <v>80.81789999999999</v>
+        <v>79.3914</v>
       </c>
       <c r="I23" t="n">
-        <v>0.653102</v>
+        <v>0.663385</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2.2538e-123</t>
+          <t>1.0501e-127</t>
         </is>
       </c>
       <c r="K23" t="n">
-        <v>94.14</v>
+        <v>94.29000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -1338,36 +1338,36 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1.395053</v>
+        <v>1.393568</v>
       </c>
       <c r="C24" t="n">
-        <v>0.913749</v>
+        <v>0.915431</v>
       </c>
       <c r="D24" t="n">
-        <v>1.051471</v>
+        <v>1.051028</v>
       </c>
       <c r="E24" t="n">
-        <v>0.864926</v>
+        <v>0.864166</v>
       </c>
       <c r="F24" t="n">
-        <v>1.296401</v>
+        <v>1.294958</v>
       </c>
       <c r="G24" t="n">
-        <v>0.887247</v>
+        <v>0.888903</v>
       </c>
       <c r="H24" t="n">
-        <v>72.0198</v>
+        <v>71.1576</v>
       </c>
       <c r="I24" t="n">
-        <v>0.611537</v>
+        <v>0.616667</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>3.1438e-142</t>
+          <t>1.5764e-144</t>
         </is>
       </c>
       <c r="K24" t="n">
-        <v>95.43000000000001</v>
+        <v>95.7</v>
       </c>
     </row>
     <row r="25">
@@ -1377,36 +1377,36 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.81828</v>
+        <v>0.802436</v>
       </c>
       <c r="C25" t="n">
-        <v>0.852904</v>
+        <v>0.8562</v>
       </c>
       <c r="D25" t="n">
-        <v>0.965545</v>
+        <v>0.964331</v>
       </c>
       <c r="E25" t="n">
-        <v>0.855844</v>
+        <v>0.85363</v>
       </c>
       <c r="F25" t="n">
-        <v>0.8597399999999999</v>
+        <v>0.848056</v>
       </c>
       <c r="G25" t="n">
-        <v>0.84215</v>
+        <v>0.844019</v>
       </c>
       <c r="H25" t="n">
-        <v>123.1902</v>
+        <v>119.6909</v>
       </c>
       <c r="I25" t="n">
-        <v>0.559666</v>
+        <v>0.559593</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>9.9146e-85</t>
+          <t>2.6999e-84</t>
         </is>
       </c>
       <c r="K25" t="n">
-        <v>95.47</v>
+        <v>95.54000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -1416,36 +1416,36 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1.0598</v>
+        <v>1.015329</v>
       </c>
       <c r="C26" t="n">
-        <v>0.83461</v>
+        <v>0.833599</v>
       </c>
       <c r="D26" t="n">
-        <v>1.037884</v>
+        <v>1.036288</v>
       </c>
       <c r="E26" t="n">
-        <v>0.835172</v>
+        <v>0.831033</v>
       </c>
       <c r="F26" t="n">
-        <v>1.052802</v>
+        <v>1.020099</v>
       </c>
       <c r="G26" t="n">
-        <v>0.820361</v>
+        <v>0.818808</v>
       </c>
       <c r="H26" t="n">
-        <v>81.2058</v>
+        <v>79.13809999999999</v>
       </c>
       <c r="I26" t="n">
-        <v>0.6043230000000001</v>
+        <v>0.6135</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>3.9602e-115</t>
+          <t>1.2567e-118</t>
         </is>
       </c>
       <c r="K26" t="n">
-        <v>94.25</v>
+        <v>94.38</v>
       </c>
     </row>
     <row r="27">
@@ -1455,36 +1455,36 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.9886779999999999</v>
+        <v>0.981196</v>
       </c>
       <c r="C27" t="n">
-        <v>0.82935</v>
+        <v>0.832407</v>
       </c>
       <c r="D27" t="n">
-        <v>1.022693</v>
+        <v>1.020451</v>
       </c>
       <c r="E27" t="n">
-        <v>0.831192</v>
+        <v>0.825798</v>
       </c>
       <c r="F27" t="n">
-        <v>0.994557</v>
+        <v>0.988649</v>
       </c>
       <c r="G27" t="n">
-        <v>0.807932</v>
+        <v>0.810428</v>
       </c>
       <c r="H27" t="n">
-        <v>92.10469999999999</v>
+        <v>88.6026</v>
       </c>
       <c r="I27" t="n">
-        <v>0.616559</v>
+        <v>0.623694</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>6.9210e-49</t>
+          <t>1.9216e-49</t>
         </is>
       </c>
       <c r="K27" t="n">
-        <v>91.19</v>
+        <v>91.93000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1494,36 +1494,36 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.629977</v>
+        <v>0.615772</v>
       </c>
       <c r="C28" t="n">
-        <v>0.774596</v>
+        <v>0.7717000000000001</v>
       </c>
       <c r="D28" t="n">
-        <v>0.93328</v>
+        <v>0.931424</v>
       </c>
       <c r="E28" t="n">
-        <v>0.773363</v>
+        <v>0.770782</v>
       </c>
       <c r="F28" t="n">
-        <v>0.7168099999999999</v>
+        <v>0.7061460000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>0.764037</v>
+        <v>0.761314</v>
       </c>
       <c r="H28" t="n">
-        <v>111.5304</v>
+        <v>107.7279</v>
       </c>
       <c r="I28" t="n">
-        <v>0.40326</v>
+        <v>0.401427</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2.0118e-70</t>
+          <t>3.6110e-69</t>
         </is>
       </c>
       <c r="K28" t="n">
-        <v>95.61</v>
+        <v>95.63</v>
       </c>
     </row>
     <row r="29">
@@ -1533,36 +1533,36 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1.030382</v>
+        <v>1.029086</v>
       </c>
       <c r="C29" t="n">
-        <v>0.84889</v>
+        <v>0.850955</v>
       </c>
       <c r="D29" t="n">
-        <v>1.042491</v>
+        <v>1.041688</v>
       </c>
       <c r="E29" t="n">
-        <v>0.836247</v>
+        <v>0.834156</v>
       </c>
       <c r="F29" t="n">
-        <v>1.031529</v>
+        <v>1.030425</v>
       </c>
       <c r="G29" t="n">
-        <v>0.825326</v>
+        <v>0.826937</v>
       </c>
       <c r="H29" t="n">
-        <v>89.7319</v>
+        <v>88.9037</v>
       </c>
       <c r="I29" t="n">
-        <v>0.608052</v>
+        <v>0.609144</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>5.0673e-59</t>
+          <t>7.0384e-59</t>
         </is>
       </c>
       <c r="K29" t="n">
-        <v>92.12</v>
+        <v>92.42</v>
       </c>
     </row>
     <row r="30">
@@ -1572,36 +1572,36 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.042619</v>
+        <v>1.032357</v>
       </c>
       <c r="C30" t="n">
-        <v>0.896451</v>
+        <v>0.896393</v>
       </c>
       <c r="D30" t="n">
-        <v>1.037079</v>
+        <v>1.034391</v>
       </c>
       <c r="E30" t="n">
-        <v>0.87492</v>
+        <v>0.869807</v>
       </c>
       <c r="F30" t="n">
-        <v>1.040759</v>
+        <v>1.032663</v>
       </c>
       <c r="G30" t="n">
-        <v>0.880762</v>
+        <v>0.879568</v>
       </c>
       <c r="H30" t="n">
-        <v>79.7085</v>
+        <v>77.0675</v>
       </c>
       <c r="I30" t="n">
-        <v>0.438577</v>
+        <v>0.440122</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>5.3623e-56</t>
+          <t>1.1315e-55</t>
         </is>
       </c>
       <c r="K30" t="n">
-        <v>96.48</v>
+        <v>96.61</v>
       </c>
     </row>
     <row r="31">
@@ -1650,36 +1650,36 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1.10001</v>
+        <v>1.096199</v>
       </c>
       <c r="C32" t="n">
-        <v>0.810926</v>
+        <v>0.81201</v>
       </c>
       <c r="D32" t="n">
-        <v>1.008935</v>
+        <v>1.008196</v>
       </c>
       <c r="E32" t="n">
-        <v>0.782892</v>
+        <v>0.78072</v>
       </c>
       <c r="F32" t="n">
-        <v>1.073291</v>
+        <v>1.070185</v>
       </c>
       <c r="G32" t="n">
-        <v>0.786494</v>
+        <v>0.787276</v>
       </c>
       <c r="H32" t="n">
-        <v>80.8921</v>
+        <v>78.6337</v>
       </c>
       <c r="I32" t="n">
-        <v>0.56959</v>
+        <v>0.57512</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>9.5295e-57</t>
+          <t>1.0247e-57</t>
         </is>
       </c>
       <c r="K32" t="n">
-        <v>93.18000000000001</v>
+        <v>93.45</v>
       </c>
     </row>
     <row r="33">
@@ -1689,36 +1689,36 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1.155154</v>
+        <v>1.15308</v>
       </c>
       <c r="C33" t="n">
-        <v>0.866048</v>
+        <v>0.867328</v>
       </c>
       <c r="D33" t="n">
-        <v>0.992935</v>
+        <v>0.992524</v>
       </c>
       <c r="E33" t="n">
-        <v>0.821245</v>
+        <v>0.820171</v>
       </c>
       <c r="F33" t="n">
-        <v>1.108583</v>
+        <v>1.106852</v>
       </c>
       <c r="G33" t="n">
-        <v>0.841792</v>
+        <v>0.842863</v>
       </c>
       <c r="H33" t="n">
-        <v>82.76739999999999</v>
+        <v>82.2414</v>
       </c>
       <c r="I33" t="n">
-        <v>0.616766</v>
+        <v>0.620484</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>5.6254e-99</t>
+          <t>4.5964e-100</t>
         </is>
       </c>
       <c r="K33" t="n">
-        <v>95.61</v>
+        <v>95.81</v>
       </c>
     </row>
     <row r="34">
@@ -1806,36 +1806,36 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1.39751</v>
+        <v>1.388016</v>
       </c>
       <c r="C36" t="n">
-        <v>0.9089429999999999</v>
+        <v>0.907519</v>
       </c>
       <c r="D36" t="n">
-        <v>1.049162</v>
+        <v>1.046878</v>
       </c>
       <c r="E36" t="n">
-        <v>0.865659</v>
+        <v>0.86121</v>
       </c>
       <c r="F36" t="n">
-        <v>1.295856</v>
+        <v>1.288244</v>
       </c>
       <c r="G36" t="n">
-        <v>0.888004</v>
+        <v>0.88608</v>
       </c>
       <c r="H36" t="n">
-        <v>70.1658</v>
+        <v>67.3908</v>
       </c>
       <c r="I36" t="n">
-        <v>0.635149</v>
+        <v>0.6417119999999999</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>1.8172e-181</t>
+          <t>1.6993e-183</t>
         </is>
       </c>
       <c r="K36" t="n">
-        <v>96.94</v>
+        <v>97.08</v>
       </c>
     </row>
     <row r="37">
@@ -1845,36 +1845,36 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.415531</v>
+        <v>0.412561</v>
       </c>
       <c r="C37" t="n">
-        <v>0.804327</v>
+        <v>0.804553</v>
       </c>
       <c r="D37" t="n">
-        <v>0.735437</v>
+        <v>0.733973</v>
       </c>
       <c r="E37" t="n">
-        <v>0.805597</v>
+        <v>0.803322</v>
       </c>
       <c r="F37" t="n">
-        <v>0.508565</v>
+        <v>0.506148</v>
       </c>
       <c r="G37" t="n">
-        <v>0.7948190000000001</v>
+        <v>0.794747</v>
       </c>
       <c r="H37" t="n">
-        <v>76.7312</v>
+        <v>74.03579999999999</v>
       </c>
       <c r="I37" t="n">
-        <v>0.016179</v>
+        <v>0.012163</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>6.0898e-01</t>
+          <t>7.0144e-01</t>
         </is>
       </c>
       <c r="K37" t="n">
-        <v>95.91</v>
+        <v>96.08</v>
       </c>
     </row>
     <row r="38">
@@ -1884,36 +1884,36 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.906529</v>
+        <v>0.883696</v>
       </c>
       <c r="C38" t="n">
-        <v>0.797629</v>
+        <v>0.7969079999999999</v>
       </c>
       <c r="D38" t="n">
-        <v>1.00977</v>
+        <v>1.004154</v>
       </c>
       <c r="E38" t="n">
-        <v>0.816405</v>
+        <v>0.807559</v>
       </c>
       <c r="F38" t="n">
-        <v>0.934602</v>
+        <v>0.916483</v>
       </c>
       <c r="G38" t="n">
-        <v>0.784265</v>
+        <v>0.781925</v>
       </c>
       <c r="H38" t="n">
-        <v>117.8059</v>
+        <v>106.9498</v>
       </c>
       <c r="I38" t="n">
-        <v>0.574637</v>
+        <v>0.593812</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>1.1245e-64</t>
+          <t>2.9144e-67</t>
         </is>
       </c>
       <c r="K38" t="n">
-        <v>92.23999999999999</v>
+        <v>92.5</v>
       </c>
     </row>
     <row r="39">
@@ -1962,36 +1962,36 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1.309326</v>
+        <v>1.308224</v>
       </c>
       <c r="C40" t="n">
-        <v>0.89655</v>
+        <v>0.897521</v>
       </c>
       <c r="D40" t="n">
-        <v>1.050057</v>
+        <v>1.049621</v>
       </c>
       <c r="E40" t="n">
-        <v>0.864142</v>
+        <v>0.863007</v>
       </c>
       <c r="F40" t="n">
-        <v>1.234077</v>
+        <v>1.233044</v>
       </c>
       <c r="G40" t="n">
-        <v>0.875546</v>
+        <v>0.876322</v>
       </c>
       <c r="H40" t="n">
-        <v>79.9383</v>
+        <v>79.28360000000001</v>
       </c>
       <c r="I40" t="n">
-        <v>0.614573</v>
+        <v>0.617859</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>6.5304e-118</t>
+          <t>4.3426e-119</t>
         </is>
       </c>
       <c r="K40" t="n">
-        <v>95.65000000000001</v>
+        <v>95.81</v>
       </c>
     </row>
     <row r="41">
@@ -2001,36 +2001,36 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1.180048</v>
+        <v>1.1767</v>
       </c>
       <c r="C41" t="n">
-        <v>0.914911</v>
+        <v>0.919071</v>
       </c>
       <c r="D41" t="n">
-        <v>0.8568519999999999</v>
+        <v>0.856016</v>
       </c>
       <c r="E41" t="n">
-        <v>0.822207</v>
+        <v>0.8217989999999999</v>
       </c>
       <c r="F41" t="n">
-        <v>1.084357</v>
+        <v>1.081208</v>
       </c>
       <c r="G41" t="n">
-        <v>0.879161</v>
+        <v>0.88247</v>
       </c>
       <c r="H41" t="n">
-        <v>101.0349</v>
+        <v>99.81659999999999</v>
       </c>
       <c r="I41" t="n">
-        <v>0.333396</v>
+        <v>0.351631</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>9.4171e-13</t>
+          <t>5.1084e-14</t>
         </is>
       </c>
       <c r="K41" t="n">
-        <v>96.78</v>
+        <v>96.98999999999999</v>
       </c>
     </row>
     <row r="42">
@@ -2040,36 +2040,36 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.939385</v>
+        <v>0.931301</v>
       </c>
       <c r="C42" t="n">
-        <v>0.825358</v>
+        <v>0.825821</v>
       </c>
       <c r="D42" t="n">
-        <v>1.005476</v>
+        <v>1.003613</v>
       </c>
       <c r="E42" t="n">
-        <v>0.821084</v>
+        <v>0.816864</v>
       </c>
       <c r="F42" t="n">
-        <v>0.956857</v>
+        <v>0.950424</v>
       </c>
       <c r="G42" t="n">
-        <v>0.807382</v>
+        <v>0.807048</v>
       </c>
       <c r="H42" t="n">
-        <v>105.9992</v>
+        <v>102.2553</v>
       </c>
       <c r="I42" t="n">
-        <v>0.617388</v>
+        <v>0.6263649999999999</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>3.4928e-77</t>
+          <t>2.7917e-79</t>
         </is>
       </c>
       <c r="K42" t="n">
-        <v>93.22</v>
+        <v>93.44</v>
       </c>
     </row>
     <row r="43">
@@ -2079,36 +2079,36 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1.287551</v>
+        <v>1.275213</v>
       </c>
       <c r="C43" t="n">
-        <v>0.879006</v>
+        <v>0.8806659999999999</v>
       </c>
       <c r="D43" t="n">
-        <v>1.020783</v>
+        <v>1.019214</v>
       </c>
       <c r="E43" t="n">
-        <v>0.841541</v>
+        <v>0.837388</v>
       </c>
       <c r="F43" t="n">
-        <v>1.210711</v>
+        <v>1.201264</v>
       </c>
       <c r="G43" t="n">
-        <v>0.856174</v>
+        <v>0.856892</v>
       </c>
       <c r="H43" t="n">
-        <v>77.9485</v>
+        <v>77.01609999999999</v>
       </c>
       <c r="I43" t="n">
-        <v>0.593822</v>
+        <v>0.598395</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>5.5151e-113</t>
+          <t>5.4867e-114</t>
         </is>
       </c>
       <c r="K43" t="n">
-        <v>95.41</v>
+        <v>95.7</v>
       </c>
     </row>
     <row r="44">
@@ -2118,36 +2118,36 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1.084127</v>
+        <v>1.060926</v>
       </c>
       <c r="C44" t="n">
-        <v>0.840476</v>
+        <v>0.839637</v>
       </c>
       <c r="D44" t="n">
-        <v>1.009774</v>
+        <v>1.006663</v>
       </c>
       <c r="E44" t="n">
-        <v>0.828771</v>
+        <v>0.820855</v>
       </c>
       <c r="F44" t="n">
-        <v>1.06124</v>
+        <v>1.043502</v>
       </c>
       <c r="G44" t="n">
-        <v>0.824178</v>
+        <v>0.822072</v>
       </c>
       <c r="H44" t="n">
-        <v>80.52509999999999</v>
+        <v>76.79049999999999</v>
       </c>
       <c r="I44" t="n">
-        <v>0.50798</v>
+        <v>0.519282</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>5.7916e-70</t>
+          <t>2.4897e-72</t>
         </is>
       </c>
       <c r="K44" t="n">
-        <v>94.86</v>
+        <v>95.16</v>
       </c>
     </row>
     <row r="45">
@@ -2196,36 +2196,36 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1.239804</v>
+        <v>1.223639</v>
       </c>
       <c r="C46" t="n">
-        <v>0.854416</v>
+        <v>0.855248</v>
       </c>
       <c r="D46" t="n">
-        <v>1.039701</v>
+        <v>1.03846</v>
       </c>
       <c r="E46" t="n">
-        <v>0.831588</v>
+        <v>0.828257</v>
       </c>
       <c r="F46" t="n">
-        <v>1.181281</v>
+        <v>1.169237</v>
       </c>
       <c r="G46" t="n">
-        <v>0.836528</v>
+        <v>0.836379</v>
       </c>
       <c r="H46" t="n">
-        <v>72.9311</v>
+        <v>71.2363</v>
       </c>
       <c r="I46" t="n">
-        <v>0.611814</v>
+        <v>0.616058</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>1.3028e-174</t>
+          <t>1.5096e-176</t>
         </is>
       </c>
       <c r="K46" t="n">
-        <v>95.58</v>
+        <v>95.67</v>
       </c>
     </row>
     <row r="47">
@@ -2235,36 +2235,36 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1.067622</v>
+        <v>1.069456</v>
       </c>
       <c r="C47" t="n">
-        <v>0.838963</v>
+        <v>0.843547</v>
       </c>
       <c r="D47" t="n">
-        <v>0.855475</v>
+        <v>0.851891</v>
       </c>
       <c r="E47" t="n">
-        <v>0.780314</v>
+        <v>0.774908</v>
       </c>
       <c r="F47" t="n">
-        <v>1.005871</v>
+        <v>1.005922</v>
       </c>
       <c r="G47" t="n">
-        <v>0.807684</v>
+        <v>0.810484</v>
       </c>
       <c r="H47" t="n">
-        <v>97.0635</v>
+        <v>92.8276</v>
       </c>
       <c r="I47" t="n">
-        <v>0.43821</v>
+        <v>0.442887</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>6.7774e-24</t>
+          <t>8.3018e-24</t>
         </is>
       </c>
       <c r="K47" t="n">
-        <v>94.15000000000001</v>
+        <v>94.64</v>
       </c>
     </row>
     <row r="48">
@@ -2274,36 +2274,36 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1.118454</v>
+        <v>1.117037</v>
       </c>
       <c r="C48" t="n">
-        <v>0.836155</v>
+        <v>0.836694</v>
       </c>
       <c r="D48" t="n">
-        <v>1.027022</v>
+        <v>1.026826</v>
       </c>
       <c r="E48" t="n">
-        <v>0.82189</v>
+        <v>0.820685</v>
       </c>
       <c r="F48" t="n">
-        <v>1.091845</v>
+        <v>1.090692</v>
       </c>
       <c r="G48" t="n">
-        <v>0.811951</v>
+        <v>0.812837</v>
       </c>
       <c r="H48" t="n">
-        <v>104.563</v>
+        <v>103.5841</v>
       </c>
       <c r="I48" t="n">
-        <v>0.5713240000000001</v>
+        <v>0.575193</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>3.1325e-44</t>
+          <t>1.3693e-44</t>
         </is>
       </c>
       <c r="K48" t="n">
-        <v>91.92</v>
+        <v>92.26000000000001</v>
       </c>
     </row>
     <row r="49">
@@ -2352,36 +2352,36 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.357119</v>
+        <v>0.350384</v>
       </c>
       <c r="C50" t="n">
-        <v>0.803998</v>
+        <v>0.8075560000000001</v>
       </c>
       <c r="D50" t="n">
-        <v>0.725054</v>
+        <v>0.72135</v>
       </c>
       <c r="E50" t="n">
-        <v>0.813196</v>
+        <v>0.809653</v>
       </c>
       <c r="F50" t="n">
-        <v>0.461849</v>
+        <v>0.456292</v>
       </c>
       <c r="G50" t="n">
-        <v>0.793593</v>
+        <v>0.7961240000000001</v>
       </c>
       <c r="H50" t="n">
-        <v>82.5346</v>
+        <v>79.83199999999999</v>
       </c>
       <c r="I50" t="n">
-        <v>0.08223900000000001</v>
+        <v>0.08047799999999999</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>4.5306e-02</t>
+          <t>5.1917e-02</t>
         </is>
       </c>
       <c r="K50" t="n">
-        <v>94.59999999999999</v>
+        <v>95.03</v>
       </c>
     </row>
     <row r="51">
@@ -2391,36 +2391,36 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1.051457</v>
+        <v>1.03828</v>
       </c>
       <c r="C51" t="n">
-        <v>0.820044</v>
+        <v>0.824993</v>
       </c>
       <c r="D51" t="n">
-        <v>0.904487</v>
+        <v>0.901387</v>
       </c>
       <c r="E51" t="n">
-        <v>0.811163</v>
+        <v>0.805993</v>
       </c>
       <c r="F51" t="n">
-        <v>1.009121</v>
+        <v>0.998382</v>
       </c>
       <c r="G51" t="n">
-        <v>0.799374</v>
+        <v>0.802617</v>
       </c>
       <c r="H51" t="n">
-        <v>101.1461</v>
+        <v>95.86020000000001</v>
       </c>
       <c r="I51" t="n">
-        <v>0.556657</v>
+        <v>0.572869</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>1.1841e-37</t>
+          <t>2.6529e-39</t>
         </is>
       </c>
       <c r="K51" t="n">
-        <v>92.59999999999999</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="52">
@@ -2469,36 +2469,36 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.806043</v>
+        <v>0.7986259999999999</v>
       </c>
       <c r="C53" t="n">
-        <v>0.757266</v>
+        <v>0.758009</v>
       </c>
       <c r="D53" t="n">
-        <v>0.990377</v>
+        <v>0.988324</v>
       </c>
       <c r="E53" t="n">
-        <v>0.784659</v>
+        <v>0.77985</v>
       </c>
       <c r="F53" t="n">
-        <v>0.8570950000000001</v>
+        <v>0.851174</v>
       </c>
       <c r="G53" t="n">
-        <v>0.74525</v>
+        <v>0.7452299999999999</v>
       </c>
       <c r="H53" t="n">
-        <v>93.5136</v>
+        <v>89.13079999999999</v>
       </c>
       <c r="I53" t="n">
-        <v>0.436314</v>
+        <v>0.43998</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>1.3734e-23</t>
+          <t>9.1222e-24</t>
         </is>
       </c>
       <c r="K53" t="n">
-        <v>91.40000000000001</v>
+        <v>91.73999999999999</v>
       </c>
     </row>
     <row r="54">
@@ -2547,10 +2547,10 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1.111264</v>
+        <v>1.111413</v>
       </c>
       <c r="C55" t="n">
-        <v>0.880772</v>
+        <v>0.881953</v>
       </c>
       <c r="D55" t="n">
         <v>1.037702</v>
@@ -2559,24 +2559,24 @@
         <v>0.855784</v>
       </c>
       <c r="F55" t="n">
-        <v>1.087391</v>
+        <v>1.087509</v>
       </c>
       <c r="G55" t="n">
-        <v>0.856779</v>
+        <v>0.857927</v>
       </c>
       <c r="H55" t="n">
-        <v>87.4752</v>
+        <v>87.587</v>
       </c>
       <c r="I55" t="n">
-        <v>0.645616</v>
+        <v>0.646164</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2.6083e-89</t>
+          <t>2.1734e-89</t>
         </is>
       </c>
       <c r="K55" t="n">
-        <v>93.56999999999999</v>
+        <v>93.7</v>
       </c>
     </row>
     <row r="56">
@@ -2586,36 +2586,36 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1.259109</v>
+        <v>1.248261</v>
       </c>
       <c r="C56" t="n">
-        <v>0.914452</v>
+        <v>0.915702</v>
       </c>
       <c r="D56" t="n">
-        <v>1.044533</v>
+        <v>1.042529</v>
       </c>
       <c r="E56" t="n">
-        <v>0.880624</v>
+        <v>0.876725</v>
       </c>
       <c r="F56" t="n">
-        <v>1.195952</v>
+        <v>1.187345</v>
       </c>
       <c r="G56" t="n">
-        <v>0.896218</v>
+        <v>0.896798</v>
       </c>
       <c r="H56" t="n">
-        <v>77.8519</v>
+        <v>75.3004</v>
       </c>
       <c r="I56" t="n">
-        <v>0.5390740000000001</v>
+        <v>0.548343</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>9.9055e-107</t>
+          <t>1.2805e-109</t>
         </is>
       </c>
       <c r="K56" t="n">
-        <v>96.94</v>
+        <v>97.26000000000001</v>
       </c>
     </row>
     <row r="57">
@@ -2625,36 +2625,36 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1.183256</v>
+        <v>1.170279</v>
       </c>
       <c r="C57" t="n">
-        <v>0.882765</v>
+        <v>0.881184</v>
       </c>
       <c r="D57" t="n">
-        <v>1.053642</v>
+        <v>1.05241</v>
       </c>
       <c r="E57" t="n">
-        <v>0.839712</v>
+        <v>0.836302</v>
       </c>
       <c r="F57" t="n">
-        <v>1.145217</v>
+        <v>1.135453</v>
       </c>
       <c r="G57" t="n">
-        <v>0.859697</v>
+        <v>0.858006</v>
       </c>
       <c r="H57" t="n">
-        <v>67.26819999999999</v>
+        <v>66.3027</v>
       </c>
       <c r="I57" t="n">
-        <v>0.617435</v>
+        <v>0.6217279999999999</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>3.8686e-113</t>
+          <t>2.7456e-114</t>
         </is>
       </c>
       <c r="K57" t="n">
-        <v>95.97</v>
+        <v>96.13</v>
       </c>
     </row>
     <row r="58">
@@ -2703,36 +2703,36 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1.028601</v>
+        <v>1.012899</v>
       </c>
       <c r="C59" t="n">
-        <v>0.828623</v>
+        <v>0.829532</v>
       </c>
       <c r="D59" t="n">
-        <v>1.014658</v>
+        <v>1.012134</v>
       </c>
       <c r="E59" t="n">
-        <v>0.8092859999999999</v>
+        <v>0.801463</v>
       </c>
       <c r="F59" t="n">
-        <v>1.023709</v>
+        <v>1.011437</v>
       </c>
       <c r="G59" t="n">
-        <v>0.810844</v>
+        <v>0.810203</v>
       </c>
       <c r="H59" t="n">
-        <v>79.34439999999999</v>
+        <v>76.803</v>
       </c>
       <c r="I59" t="n">
-        <v>0.5612470000000001</v>
+        <v>0.577756</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>1.6397e-88</t>
+          <t>2.7231e-93</t>
         </is>
       </c>
       <c r="K59" t="n">
-        <v>95.06999999999999</v>
+        <v>95.45999999999999</v>
       </c>
     </row>
     <row r="60">
@@ -2742,36 +2742,36 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1.315708</v>
+        <v>1.306837</v>
       </c>
       <c r="C60" t="n">
-        <v>0.8836619999999999</v>
+        <v>0.883663</v>
       </c>
       <c r="D60" t="n">
-        <v>1.055648</v>
+        <v>1.053596</v>
       </c>
       <c r="E60" t="n">
-        <v>0.850263</v>
+        <v>0.845523</v>
       </c>
       <c r="F60" t="n">
-        <v>1.240168</v>
+        <v>1.233083</v>
       </c>
       <c r="G60" t="n">
-        <v>0.862768</v>
+        <v>0.86183</v>
       </c>
       <c r="H60" t="n">
-        <v>68.94119999999999</v>
+        <v>66.8005</v>
       </c>
       <c r="I60" t="n">
-        <v>0.648911</v>
+        <v>0.653641</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>3.0600e-166</t>
+          <t>2.1445e-167</t>
         </is>
       </c>
       <c r="K60" t="n">
-        <v>95.73999999999999</v>
+        <v>95.90000000000001</v>
       </c>
     </row>
     <row r="61">
@@ -2820,36 +2820,36 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1.206599</v>
+        <v>1.193641</v>
       </c>
       <c r="C62" t="n">
-        <v>0.85488</v>
+        <v>0.854443</v>
       </c>
       <c r="D62" t="n">
-        <v>1.033082</v>
+        <v>1.030099</v>
       </c>
       <c r="E62" t="n">
-        <v>0.838372</v>
+        <v>0.83187</v>
       </c>
       <c r="F62" t="n">
-        <v>1.156413</v>
+        <v>1.146248</v>
       </c>
       <c r="G62" t="n">
-        <v>0.8391690000000001</v>
+        <v>0.837515</v>
       </c>
       <c r="H62" t="n">
-        <v>69.39490000000001</v>
+        <v>66.2214</v>
       </c>
       <c r="I62" t="n">
-        <v>0.606276</v>
+        <v>0.614703</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>1.3782e-106</t>
+          <t>2.8748e-108</t>
         </is>
       </c>
       <c r="K62" t="n">
-        <v>95.72</v>
+        <v>95.93000000000001</v>
       </c>
     </row>
     <row r="63">
@@ -2859,36 +2859,36 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.864053</v>
+        <v>0.856952</v>
       </c>
       <c r="C63" t="n">
-        <v>0.79879</v>
+        <v>0.8013749999999999</v>
       </c>
       <c r="D63" t="n">
-        <v>0.997479</v>
+        <v>0.995348</v>
       </c>
       <c r="E63" t="n">
-        <v>0.80257</v>
+        <v>0.7976259999999999</v>
       </c>
       <c r="F63" t="n">
-        <v>0.900397</v>
+        <v>0.894627</v>
       </c>
       <c r="G63" t="n">
-        <v>0.783663</v>
+        <v>0.784776</v>
       </c>
       <c r="H63" t="n">
-        <v>88.2497</v>
+        <v>84.53230000000001</v>
       </c>
       <c r="I63" t="n">
-        <v>0.557813</v>
+        <v>0.570545</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>3.4724e-70</t>
+          <t>2.8148e-73</t>
         </is>
       </c>
       <c r="K63" t="n">
-        <v>93.25</v>
+        <v>93.53</v>
       </c>
     </row>
     <row r="64">
@@ -2898,36 +2898,36 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1.061469</v>
+        <v>1.049551</v>
       </c>
       <c r="C64" t="n">
-        <v>0.857883</v>
+        <v>0.8591569999999999</v>
       </c>
       <c r="D64" t="n">
-        <v>0.991642</v>
+        <v>0.988753</v>
       </c>
       <c r="E64" t="n">
-        <v>0.835475</v>
+        <v>0.828164</v>
       </c>
       <c r="F64" t="n">
-        <v>1.039835</v>
+        <v>1.03032</v>
       </c>
       <c r="G64" t="n">
-        <v>0.84195</v>
+        <v>0.841553</v>
       </c>
       <c r="H64" t="n">
-        <v>86.5065</v>
+        <v>82.84180000000001</v>
       </c>
       <c r="I64" t="n">
-        <v>0.618142</v>
+        <v>0.62727</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>5.2118e-110</t>
+          <t>2.5057e-112</t>
         </is>
       </c>
       <c r="K64" t="n">
-        <v>96.31999999999999</v>
+        <v>96.66</v>
       </c>
     </row>
     <row r="65">
@@ -2937,36 +2937,36 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1.054863</v>
+        <v>1.009243</v>
       </c>
       <c r="C65" t="n">
-        <v>0.822672</v>
+        <v>0.82455</v>
       </c>
       <c r="D65" t="n">
-        <v>1.031138</v>
+        <v>1.029031</v>
       </c>
       <c r="E65" t="n">
-        <v>0.807225</v>
+        <v>0.801679</v>
       </c>
       <c r="F65" t="n">
-        <v>1.046719</v>
+        <v>1.013277</v>
       </c>
       <c r="G65" t="n">
-        <v>0.806245</v>
+        <v>0.806406</v>
       </c>
       <c r="H65" t="n">
-        <v>77.68729999999999</v>
+        <v>76.0707</v>
       </c>
       <c r="I65" t="n">
-        <v>0.608393</v>
+        <v>0.59566</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>1.6238e-90</t>
+          <t>4.7774e-85</t>
         </is>
       </c>
       <c r="K65" t="n">
-        <v>95.13</v>
+        <v>95.31</v>
       </c>
     </row>
     <row r="66">
@@ -2976,36 +2976,36 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.830162</v>
+        <v>0.808215</v>
       </c>
       <c r="C66" t="n">
-        <v>0.757874</v>
+        <v>0.7550249999999999</v>
       </c>
       <c r="D66" t="n">
-        <v>0.964004</v>
+        <v>0.957602</v>
       </c>
       <c r="E66" t="n">
-        <v>0.77286</v>
+        <v>0.76093</v>
       </c>
       <c r="F66" t="n">
-        <v>0.869971</v>
+        <v>0.852295</v>
       </c>
       <c r="G66" t="n">
-        <v>0.75136</v>
+        <v>0.747244</v>
       </c>
       <c r="H66" t="n">
-        <v>110.8693</v>
+        <v>103.2274</v>
       </c>
       <c r="I66" t="n">
-        <v>0.540447</v>
+        <v>0.560069</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>1.5294e-55</t>
+          <t>1.7906e-58</t>
         </is>
       </c>
       <c r="K66" t="n">
-        <v>95.25</v>
+        <v>95.81999999999999</v>
       </c>
     </row>
     <row r="67">
@@ -3015,36 +3015,36 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1.020707</v>
+        <v>1.022649</v>
       </c>
       <c r="C67" t="n">
-        <v>0.817703</v>
+        <v>0.819698</v>
       </c>
       <c r="D67" t="n">
-        <v>0.911345</v>
+        <v>0.9108309999999999</v>
       </c>
       <c r="E67" t="n">
-        <v>0.796899</v>
+        <v>0.795833</v>
       </c>
       <c r="F67" t="n">
-        <v>0.9884309999999999</v>
+        <v>0.98939</v>
       </c>
       <c r="G67" t="n">
-        <v>0.799714</v>
+        <v>0.801821</v>
       </c>
       <c r="H67" t="n">
-        <v>106.4997</v>
+        <v>103.313</v>
       </c>
       <c r="I67" t="n">
-        <v>0.571013</v>
+        <v>0.5821229999999999</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>1.2903e-71</t>
+          <t>6.3057e-74</t>
         </is>
       </c>
       <c r="K67" t="n">
-        <v>95.09</v>
+        <v>95.51000000000001</v>
       </c>
     </row>
     <row r="68">
@@ -3054,36 +3054,36 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.988397</v>
+        <v>0.970619</v>
       </c>
       <c r="C68" t="n">
-        <v>0.790734</v>
+        <v>0.791774</v>
       </c>
       <c r="D68" t="n">
-        <v>1.019152</v>
+        <v>1.014122</v>
       </c>
       <c r="E68" t="n">
-        <v>0.808187</v>
+        <v>0.79675</v>
       </c>
       <c r="F68" t="n">
-        <v>0.994849</v>
+        <v>0.980339</v>
       </c>
       <c r="G68" t="n">
-        <v>0.77854</v>
+        <v>0.777701</v>
       </c>
       <c r="H68" t="n">
-        <v>81.5393</v>
+        <v>77.14660000000001</v>
       </c>
       <c r="I68" t="n">
-        <v>0.638686</v>
+        <v>0.658215</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>5.8715e-108</t>
+          <t>1.3757e-113</t>
         </is>
       </c>
       <c r="K68" t="n">
-        <v>92.81</v>
+        <v>93.48999999999999</v>
       </c>
     </row>
     <row r="69">
@@ -3171,36 +3171,36 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.994344</v>
+        <v>0.972473</v>
       </c>
       <c r="C71" t="n">
-        <v>0.797068</v>
+        <v>0.795548</v>
       </c>
       <c r="D71" t="n">
-        <v>1.00889</v>
+        <v>1.003712</v>
       </c>
       <c r="E71" t="n">
-        <v>0.790639</v>
+        <v>0.778844</v>
       </c>
       <c r="F71" t="n">
-        <v>0.9982220000000001</v>
+        <v>0.980778</v>
       </c>
       <c r="G71" t="n">
-        <v>0.779185</v>
+        <v>0.775766</v>
       </c>
       <c r="H71" t="n">
-        <v>80.3073</v>
+        <v>74.97709999999999</v>
       </c>
       <c r="I71" t="n">
-        <v>0.566697</v>
+        <v>0.577887</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>6.5048e-77</t>
+          <t>1.1773e-78</t>
         </is>
       </c>
       <c r="K71" t="n">
-        <v>93.27</v>
+        <v>93.68000000000001</v>
       </c>
     </row>
     <row r="72">
@@ -3210,36 +3210,36 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1.185506</v>
+        <v>1.176328</v>
       </c>
       <c r="C72" t="n">
-        <v>0.9012289999999999</v>
+        <v>0.904014</v>
       </c>
       <c r="D72" t="n">
-        <v>0.974032</v>
+        <v>0.972867</v>
       </c>
       <c r="E72" t="n">
-        <v>0.865648</v>
+        <v>0.862523</v>
       </c>
       <c r="F72" t="n">
-        <v>1.124857</v>
+        <v>1.117727</v>
       </c>
       <c r="G72" t="n">
-        <v>0.869875</v>
+        <v>0.871737</v>
       </c>
       <c r="H72" t="n">
-        <v>95.377</v>
+        <v>93.88549999999999</v>
       </c>
       <c r="I72" t="n">
-        <v>0.558728</v>
+        <v>0.559283</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>1.1710e-45</t>
+          <t>2.3559e-45</t>
         </is>
       </c>
       <c r="K72" t="n">
-        <v>92.04000000000001</v>
+        <v>92.34</v>
       </c>
     </row>
     <row r="73">
@@ -3249,36 +3249,36 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.772949</v>
+        <v>0.739116</v>
       </c>
       <c r="C73" t="n">
-        <v>0.820628</v>
+        <v>0.817313</v>
       </c>
       <c r="D73" t="n">
-        <v>0.814927</v>
+        <v>0.808159</v>
       </c>
       <c r="E73" t="n">
-        <v>0.8110540000000001</v>
+        <v>0.804131</v>
       </c>
       <c r="F73" t="n">
-        <v>0.786114</v>
+        <v>0.760015</v>
       </c>
       <c r="G73" t="n">
-        <v>0.8111</v>
+        <v>0.807069</v>
       </c>
       <c r="H73" t="n">
-        <v>82.4987</v>
+        <v>79.3935</v>
       </c>
       <c r="I73" t="n">
-        <v>0.317704</v>
+        <v>0.311092</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>3.5753e-55</t>
+          <t>5.6950e-52</t>
         </is>
       </c>
       <c r="K73" t="n">
-        <v>97.26000000000001</v>
+        <v>97.39</v>
       </c>
     </row>
     <row r="74">
@@ -3288,36 +3288,36 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1.134264</v>
+        <v>1.118829</v>
       </c>
       <c r="C74" t="n">
-        <v>0.882812</v>
+        <v>0.881652</v>
       </c>
       <c r="D74" t="n">
-        <v>1.025796</v>
+        <v>1.02302</v>
       </c>
       <c r="E74" t="n">
-        <v>0.850342</v>
+        <v>0.844611</v>
       </c>
       <c r="F74" t="n">
-        <v>1.102203</v>
+        <v>1.090348</v>
       </c>
       <c r="G74" t="n">
-        <v>0.864306</v>
+        <v>0.862102</v>
       </c>
       <c r="H74" t="n">
-        <v>73.0248</v>
+        <v>70.4935</v>
       </c>
       <c r="I74" t="n">
-        <v>0.508871</v>
+        <v>0.509448</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>7.7794e-131</t>
+          <t>2.0646e-129</t>
         </is>
       </c>
       <c r="K74" t="n">
-        <v>96.56</v>
+        <v>96.67</v>
       </c>
     </row>
     <row r="75">
@@ -3366,36 +3366,36 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1.217639</v>
+        <v>1.217994</v>
       </c>
       <c r="C76" t="n">
-        <v>0.909524</v>
+        <v>0.911155</v>
       </c>
       <c r="D76" t="n">
-        <v>1.071689</v>
+        <v>1.071767</v>
       </c>
       <c r="E76" t="n">
-        <v>0.904235</v>
+        <v>0.905735</v>
       </c>
       <c r="F76" t="n">
-        <v>1.17511</v>
+        <v>1.175396</v>
       </c>
       <c r="G76" t="n">
-        <v>0.886891</v>
+        <v>0.888772</v>
       </c>
       <c r="H76" t="n">
-        <v>96.9149</v>
+        <v>96.50879999999999</v>
       </c>
       <c r="I76" t="n">
-        <v>0.553514</v>
+        <v>0.553687</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>7.2534e-48</t>
+          <t>1.3974e-47</t>
         </is>
       </c>
       <c r="K76" t="n">
-        <v>92.23999999999999</v>
+        <v>92.36</v>
       </c>
     </row>
     <row r="77">
@@ -3444,36 +3444,36 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1.040046</v>
+        <v>0.9808249999999999</v>
       </c>
       <c r="C78" t="n">
-        <v>0.853159</v>
+        <v>0.853679</v>
       </c>
       <c r="D78" t="n">
-        <v>0.987693</v>
+        <v>0.983884</v>
       </c>
       <c r="E78" t="n">
-        <v>0.8485780000000001</v>
+        <v>0.837829</v>
       </c>
       <c r="F78" t="n">
-        <v>1.024394</v>
+        <v>0.980086</v>
       </c>
       <c r="G78" t="n">
-        <v>0.832088</v>
+        <v>0.830754</v>
       </c>
       <c r="H78" t="n">
-        <v>96.39100000000001</v>
+        <v>91.9697</v>
       </c>
       <c r="I78" t="n">
-        <v>0.55969</v>
+        <v>0.599322</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>1.0034e-57</t>
+          <t>5.5033e-66</t>
         </is>
       </c>
       <c r="K78" t="n">
-        <v>92.26000000000001</v>
+        <v>92.77</v>
       </c>
     </row>
     <row r="79">
@@ -3483,36 +3483,36 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>1.2596</v>
+        <v>1.240955</v>
       </c>
       <c r="C79" t="n">
-        <v>0.854808</v>
+        <v>0.854901</v>
       </c>
       <c r="D79" t="n">
-        <v>1.052677</v>
+        <v>1.051003</v>
       </c>
       <c r="E79" t="n">
-        <v>0.824204</v>
+        <v>0.819377</v>
       </c>
       <c r="F79" t="n">
-        <v>1.199345</v>
+        <v>1.185328</v>
       </c>
       <c r="G79" t="n">
-        <v>0.8367520000000001</v>
+        <v>0.835876</v>
       </c>
       <c r="H79" t="n">
-        <v>67.5035</v>
+        <v>65.13720000000001</v>
       </c>
       <c r="I79" t="n">
-        <v>0.635191</v>
+        <v>0.640962</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>3.3940e-205</t>
+          <t>6.7931e-208</t>
         </is>
       </c>
       <c r="K79" t="n">
-        <v>96.41</v>
+        <v>96.59999999999999</v>
       </c>
     </row>
     <row r="80">
@@ -3522,36 +3522,36 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.8740289999999999</v>
+        <v>0.82579</v>
       </c>
       <c r="C80" t="n">
-        <v>0.798866</v>
+        <v>0.793817</v>
       </c>
       <c r="D80" t="n">
-        <v>1.006321</v>
+        <v>1.001457</v>
       </c>
       <c r="E80" t="n">
-        <v>0.811286</v>
+        <v>0.799424</v>
       </c>
       <c r="F80" t="n">
-        <v>0.90983</v>
+        <v>0.873342</v>
       </c>
       <c r="G80" t="n">
-        <v>0.785181</v>
+        <v>0.778689</v>
       </c>
       <c r="H80" t="n">
-        <v>95.5432</v>
+        <v>92.444</v>
       </c>
       <c r="I80" t="n">
-        <v>0.530563</v>
+        <v>0.53432</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>5.5923e-49</t>
+          <t>1.1230e-48</t>
         </is>
       </c>
       <c r="K80" t="n">
-        <v>92.84999999999999</v>
+        <v>92.98999999999999</v>
       </c>
     </row>
     <row r="81">
@@ -3561,36 +3561,36 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.855056</v>
+        <v>0.849144</v>
       </c>
       <c r="C81" t="n">
-        <v>0.758646</v>
+        <v>0.7604880000000001</v>
       </c>
       <c r="D81" t="n">
-        <v>1.008941</v>
+        <v>1.007517</v>
       </c>
       <c r="E81" t="n">
-        <v>0.804464</v>
+        <v>0.800737</v>
       </c>
       <c r="F81" t="n">
-        <v>0.897661</v>
+        <v>0.892875</v>
       </c>
       <c r="G81" t="n">
-        <v>0.7503</v>
+        <v>0.751219</v>
       </c>
       <c r="H81" t="n">
-        <v>115.9955</v>
+        <v>114.147</v>
       </c>
       <c r="I81" t="n">
-        <v>0.505213</v>
+        <v>0.5158199999999999</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>7.8020e-39</t>
+          <t>2.4305e-40</t>
         </is>
       </c>
       <c r="K81" t="n">
-        <v>90.84999999999999</v>
+        <v>91.11</v>
       </c>
     </row>
     <row r="82">
@@ -3600,36 +3600,36 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.703936</v>
+        <v>0.619661</v>
       </c>
       <c r="C82" t="n">
-        <v>0.7618740000000001</v>
+        <v>0.7651019999999999</v>
       </c>
       <c r="D82" t="n">
-        <v>0.934069</v>
+        <v>0.932944</v>
       </c>
       <c r="E82" t="n">
-        <v>0.771938</v>
+        <v>0.770844</v>
       </c>
       <c r="F82" t="n">
-        <v>0.767977</v>
+        <v>0.706947</v>
       </c>
       <c r="G82" t="n">
-        <v>0.748318</v>
+        <v>0.750844</v>
       </c>
       <c r="H82" t="n">
-        <v>105.0635</v>
+        <v>99.79510000000001</v>
       </c>
       <c r="I82" t="n">
-        <v>0.407259</v>
+        <v>0.388027</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>6.3881e-41</t>
+          <t>1.0407e-36</t>
         </is>
       </c>
       <c r="K82" t="n">
-        <v>92.84</v>
+        <v>93.09</v>
       </c>
     </row>
     <row r="83">
@@ -3678,36 +3678,36 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.981195</v>
+        <v>0.955593</v>
       </c>
       <c r="C84" t="n">
-        <v>0.806993</v>
+        <v>0.806388</v>
       </c>
       <c r="D84" t="n">
-        <v>1.027048</v>
+        <v>1.025057</v>
       </c>
       <c r="E84" t="n">
-        <v>0.817048</v>
+        <v>0.81198</v>
       </c>
       <c r="F84" t="n">
-        <v>0.99225</v>
+        <v>0.973047</v>
       </c>
       <c r="G84" t="n">
-        <v>0.795717</v>
+        <v>0.7944329999999999</v>
       </c>
       <c r="H84" t="n">
-        <v>89.3014</v>
+        <v>87.8159</v>
       </c>
       <c r="I84" t="n">
-        <v>0.605135</v>
+        <v>0.605038</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>9.3673e-70</t>
+          <t>4.9456e-69</t>
         </is>
       </c>
       <c r="K84" t="n">
-        <v>94.17</v>
+        <v>94.40000000000001</v>
       </c>
     </row>
     <row r="85">
@@ -3795,36 +3795,36 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1.148021</v>
+        <v>1.148284</v>
       </c>
       <c r="C87" t="n">
-        <v>0.879624</v>
+        <v>0.881053</v>
       </c>
       <c r="D87" t="n">
-        <v>1.049675</v>
+        <v>1.049639</v>
       </c>
       <c r="E87" t="n">
-        <v>0.857174</v>
+        <v>0.858141</v>
       </c>
       <c r="F87" t="n">
-        <v>1.118795</v>
+        <v>1.118987</v>
       </c>
       <c r="G87" t="n">
-        <v>0.858642</v>
+        <v>0.860196</v>
       </c>
       <c r="H87" t="n">
-        <v>88.45050000000001</v>
+        <v>88.0964</v>
       </c>
       <c r="I87" t="n">
-        <v>0.615061</v>
+        <v>0.615943</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>2.3572e-76</t>
+          <t>3.2663e-76</t>
         </is>
       </c>
       <c r="K87" t="n">
-        <v>94.45999999999999</v>
+        <v>94.56999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>